<commit_message>
Regenerate call sheets on ZIP-population reach
build_call_list.py now uses ZIP population when zips.csv carries it, falling back to
county population otherwise — the same basis rebuild_queue uses, so the sheet and
the database rank identically instead of drifting.

Effect on week one is small: the same 16 organizations, same numbers, three rows
moving. The two Dallas providers pass Alamo Area COG, which the county-population
basis had ahead of them. ZIP counts also drop across the board now that the 5%
residential-share threshold is applied — Community Council of Greater Dallas from
151 to 86, for instance, which is the phantom coverage the area proxy was inventing.

Adds scripts/build_call_sheet_xlsx.py so the formatted workbook is reproducible
rather than a one-off. Safe to regenerate: no capture cells were filled.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KNf8cEiheT4kiGSZPtQBi7
</commit_message>
<xml_diff>
--- a/data/call-sheets/CornerHelp-Week1-CallSheet.xlsx
+++ b/data/call-sheets/CornerHelp-Week1-CallSheet.xlsx
@@ -146,6 +146,21 @@
     <t xml:space="preserve">Collin, Denton, Grayson</t>
   </si>
   <si>
+    <t xml:space="preserve">Community Council of Greater Dallas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">+12148715065</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dallas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dallas County Department of Health and Human Services</t>
+  </si>
+  <si>
+    <t xml:space="preserve">+12148191848</t>
+  </si>
+  <si>
     <t xml:space="preserve">Alamo Area Council of Governments</t>
   </si>
   <si>
@@ -156,21 +171,6 @@
   </si>
   <si>
     <t xml:space="preserve">Bexar, Comal, Guadalupe</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Community Council of Greater Dallas</t>
-  </si>
-  <si>
-    <t xml:space="preserve">+12148715065</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Dallas</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Dallas County Department of Health and Human Services</t>
-  </si>
-  <si>
-    <t xml:space="preserve">+12148191848</t>
   </si>
   <si>
     <t xml:space="preserve">Fort Worth, City of, Neighborhood Services Department</t>
@@ -1184,7 +1184,7 @@
         <v>3</v>
       </c>
       <c r="G4" s="8" t="n">
-        <v>5789933</v>
+        <v>5745696</v>
       </c>
       <c r="H4" s="7" t="s">
         <v>29</v>
@@ -1224,7 +1224,7 @@
         <v>3</v>
       </c>
       <c r="G5" s="12" t="n">
-        <v>5789933</v>
+        <v>5745696</v>
       </c>
       <c r="H5" s="11" t="s">
         <v>29</v>
@@ -1264,7 +1264,7 @@
         <v>10</v>
       </c>
       <c r="G6" s="8" t="n">
-        <v>3254583</v>
+        <v>3014259</v>
       </c>
       <c r="H6" s="7" t="s">
         <v>35</v>
@@ -1304,7 +1304,7 @@
         <v>19</v>
       </c>
       <c r="G7" s="12" t="n">
-        <v>3107798</v>
+        <v>2952512</v>
       </c>
       <c r="H7" s="11" t="s">
         <v>39</v>
@@ -1341,13 +1341,13 @@
         <v>42</v>
       </c>
       <c r="F8" s="6" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="G8" s="8" t="n">
-        <v>2879722</v>
+        <v>2823843</v>
       </c>
       <c r="H8" s="7" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="I8" s="9"/>
       <c r="J8" s="9"/>
@@ -1369,25 +1369,25 @@
         <v>6</v>
       </c>
       <c r="B9" s="11" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C9" s="11" t="s">
         <v>26</v>
       </c>
       <c r="D9" s="10" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="E9" s="10" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="F9" s="10" t="n">
         <v>1</v>
       </c>
       <c r="G9" s="12" t="n">
-        <v>2656028</v>
+        <v>2823843</v>
       </c>
       <c r="H9" s="11" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="I9" s="9"/>
       <c r="J9" s="9"/>
@@ -1409,25 +1409,25 @@
         <v>7</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="C10" s="7" t="s">
         <v>26</v>
       </c>
       <c r="D10" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="E10" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="F10" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="G10" s="8" t="n">
+        <v>2679447</v>
+      </c>
+      <c r="H10" s="7" t="s">
         <v>48</v>
-      </c>
-      <c r="E10" s="6" t="s">
-        <v>46</v>
-      </c>
-      <c r="F10" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="G10" s="8" t="n">
-        <v>2656028</v>
-      </c>
-      <c r="H10" s="7" t="s">
-        <v>46</v>
       </c>
       <c r="I10" s="9"/>
       <c r="J10" s="9"/>
@@ -1464,7 +1464,7 @@
         <v>1</v>
       </c>
       <c r="G11" s="12" t="n">
-        <v>2230708</v>
+        <v>2373979</v>
       </c>
       <c r="H11" s="11" t="s">
         <v>52</v>
@@ -1498,13 +1498,13 @@
         <v>54</v>
       </c>
       <c r="E12" s="6" t="s">
-        <v>42</v>
+        <v>47</v>
       </c>
       <c r="F12" s="6" t="n">
         <v>1</v>
       </c>
       <c r="G12" s="8" t="n">
-        <v>2127737</v>
+        <v>2107424</v>
       </c>
       <c r="H12" s="7" t="s">
         <v>55</v>
@@ -1538,13 +1538,13 @@
         <v>57</v>
       </c>
       <c r="E13" s="10" t="s">
-        <v>42</v>
+        <v>47</v>
       </c>
       <c r="F13" s="10" t="n">
         <v>1</v>
       </c>
       <c r="G13" s="12" t="n">
-        <v>2127737</v>
+        <v>2107424</v>
       </c>
       <c r="H13" s="11" t="s">
         <v>55</v>
@@ -1584,7 +1584,7 @@
         <v>14</v>
       </c>
       <c r="G14" s="8" t="n">
-        <v>1913209</v>
+        <v>1891352</v>
       </c>
       <c r="H14" s="7" t="s">
         <v>61</v>
@@ -1624,7 +1624,7 @@
         <v>10</v>
       </c>
       <c r="G15" s="12" t="n">
-        <v>1571177</v>
+        <v>1670147</v>
       </c>
       <c r="H15" s="11" t="s">
         <v>65</v>
@@ -1664,7 +1664,7 @@
         <v>1</v>
       </c>
       <c r="G16" s="8" t="n">
-        <v>1363767</v>
+        <v>1642866</v>
       </c>
       <c r="H16" s="7" t="s">
         <v>69</v>
@@ -1704,7 +1704,7 @@
         <v>1</v>
       </c>
       <c r="G17" s="12" t="n">
-        <v>1363767</v>
+        <v>1642866</v>
       </c>
       <c r="H17" s="11" t="s">
         <v>69</v>
@@ -1744,7 +1744,7 @@
         <v>1</v>
       </c>
       <c r="G18" s="8" t="n">
-        <v>914820</v>
+        <v>869184</v>
       </c>
       <c r="H18" s="7" t="s">
         <v>75</v>
@@ -1784,7 +1784,7 @@
         <v>1</v>
       </c>
       <c r="G19" s="12" t="n">
-        <v>875784</v>
+        <v>865588</v>
       </c>
       <c r="H19" s="11" t="s">
         <v>78</v>

</xml_diff>